<commit_message>
Mise à jour des paramètres jusqu'en 2026
</commit_message>
<xml_diff>
--- a/srpp/params/qpp_history.xlsx
+++ b/srpp/params/qpp_history.xlsx
@@ -8,18 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\80002036\Documents\GitHub\srpp\srpp\params\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0576D8A-6C05-4FBC-B52A-82CC44506DDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E23D96F-BD6B-49FF-8162-2F4D8E269C44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3500" yWindow="14290" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="qppyear" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" calcOnSave="0" concurrentCalc="0"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
-      <x14:workbookPr defaultImageDpi="32767"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -27,10 +24,9 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
-      <mx:ArchID Flags="2"/>
     </ext>
   </extLst>
 </workbook>
@@ -48,6 +44,18 @@
     <t>exempt</t>
   </si>
   <si>
+    <t>worker</t>
+  </si>
+  <si>
+    <t>employer</t>
+  </si>
+  <si>
+    <t>selfemp</t>
+  </si>
+  <si>
+    <t>ca</t>
+  </si>
+  <si>
     <t>arf</t>
   </si>
   <si>
@@ -63,15 +71,6 @@
     <t>droprate</t>
   </si>
   <si>
-    <t>worker</t>
-  </si>
-  <si>
-    <t>employer</t>
-  </si>
-  <si>
-    <t>selfemp</t>
-  </si>
-  <si>
     <t>era</t>
   </si>
   <si>
@@ -84,10 +83,10 @@
     <t>supp</t>
   </si>
   <si>
-    <t>disab_base</t>
+    <t>disab_rate</t>
   </si>
   <si>
-    <t>disab_rate</t>
+    <t>disab_base</t>
   </si>
   <si>
     <t>cola</t>
@@ -120,9 +119,6 @@
     <t>reprate_s2</t>
   </si>
   <si>
-    <t>ca</t>
-  </si>
-  <si>
     <t>supp_s1</t>
   </si>
   <si>
@@ -137,137 +133,10 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri Light"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="12"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -295,188 +164,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -484,222 +180,33 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="44">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="44">
-    <cellStyle name="20 % - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20 % - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40 % - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60 % - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Avertissement" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Calcul" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Cellule liée" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Entrée" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Insatisfaisant" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Lien hypertexte" xfId="42" builtinId="8" hidden="1"/>
-    <cellStyle name="Lien hypertexte visité" xfId="43" builtinId="9" hidden="1"/>
-    <cellStyle name="Neutre" xfId="8" builtinId="28" customBuiltin="1"/>
+  <cellStyles count="3">
+    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="Lien hypertexte visité" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Satisfaisant" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Sortie" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Texte explicatif" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Titre" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Titre 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Titre 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Titre 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Titre 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Vérification" xfId="13" builtinId="23" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1011,7 +518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD61"/>
+  <dimension ref="A1:AD62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.875" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="22" max="22" width="10.875" customWidth="1"/>
@@ -1028,79 +535,79 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="G1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" t="s">
-        <v>6</v>
-      </c>
       <c r="L1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q1" t="s">
         <v>16</v>
       </c>
       <c r="R1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="S1" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="12" t="s">
+      <c r="T1" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="V1" s="12" t="s">
+      <c r="U1" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="12" t="s">
+      <c r="V1" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="12" t="s">
+      <c r="W1" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="Y1" s="12" t="s">
+      <c r="X1" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="Z1" s="12" t="s">
+      <c r="Y1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="AA1" s="11" t="s">
+      <c r="Z1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="AB1" s="11" t="s">
+      <c r="AA1" s="8" t="s">
         <v>26</v>
+      </c>
+      <c r="AB1" s="8" t="s">
+        <v>27</v>
       </c>
       <c r="AC1" t="s">
         <v>28</v>
@@ -1126,7 +633,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
       <c r="F2" s="4">
-        <f>D2+E2</f>
+        <f t="shared" ref="F2:F33" si="0">D2+E2</f>
         <v>3.5999999999999997E-2</v>
       </c>
       <c r="G2" s="4">
@@ -1219,7 +726,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
       <c r="F3" s="4">
-        <f t="shared" ref="F3:F54" si="0">D3+E3</f>
+        <f t="shared" si="0"/>
         <v>3.5999999999999997E-2</v>
       </c>
       <c r="G3" s="4">
@@ -2003,7 +1510,7 @@
         <v>106.26</v>
       </c>
       <c r="S11">
-        <v>0.10400000000000001</v>
+        <v>0.104</v>
       </c>
       <c r="T11" s="2">
         <v>1</v>
@@ -2096,7 +1603,7 @@
         <v>114.96</v>
       </c>
       <c r="S12">
-        <v>0.11199999999999999</v>
+        <v>0.112</v>
       </c>
       <c r="T12" s="2">
         <v>1</v>
@@ -2654,7 +2161,7 @@
         <v>201.44</v>
       </c>
       <c r="S18">
-        <v>0.12300000000000001</v>
+        <v>0.123</v>
       </c>
       <c r="T18" s="2">
         <v>1</v>
@@ -2747,7 +2254,7 @@
         <v>214.94</v>
       </c>
       <c r="S19">
-        <v>0.11199999999999999</v>
+        <v>0.112</v>
       </c>
       <c r="T19" s="2">
         <v>1</v>
@@ -2933,7 +2440,7 @@
         <v>233.4</v>
       </c>
       <c r="S21">
-        <v>4.4000000000000004E-2</v>
+        <v>4.3999999999999997E-2</v>
       </c>
       <c r="T21" s="2">
         <v>1</v>
@@ -3119,7 +2626,7 @@
         <v>253.64</v>
       </c>
       <c r="S23">
-        <v>4.0999999999999995E-2</v>
+        <v>4.0999999999999988E-2</v>
       </c>
       <c r="T23" s="2">
         <v>1</v>
@@ -3212,7 +2719,7 @@
         <v>264.04000000000002</v>
       </c>
       <c r="S24">
-        <v>4.4000000000000004E-2</v>
+        <v>4.3999999999999997E-2</v>
       </c>
       <c r="T24" s="2">
         <v>1</v>
@@ -3305,7 +2812,7 @@
         <v>276.70999999999998</v>
       </c>
       <c r="S25">
-        <v>4.0999999999999995E-2</v>
+        <v>4.0999999999999988E-2</v>
       </c>
       <c r="T25" s="2">
         <v>1</v>
@@ -3584,7 +3091,7 @@
         <v>312.33</v>
       </c>
       <c r="S28">
-        <v>5.7999999999999996E-2</v>
+        <v>5.8000000000000003E-2</v>
       </c>
       <c r="T28" s="2">
         <v>1</v>
@@ -3677,7 +3184,7 @@
         <v>318.26</v>
       </c>
       <c r="S29">
-        <v>1.8000000000000002E-2</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="T29" s="2">
         <v>1</v>
@@ -4102,7 +3609,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
       <c r="F34" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="F34:F65" si="1">D34+E34</f>
         <v>6.4000000000000001E-2</v>
       </c>
       <c r="G34" s="4">
@@ -4195,7 +3702,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
       <c r="F35" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="G35" s="4">
@@ -4288,7 +3795,7 @@
         <v>3.9E-2</v>
       </c>
       <c r="F36" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>7.8E-2</v>
       </c>
       <c r="G36" s="4">
@@ -4381,7 +3888,7 @@
         <v>4.2999999999999997E-2</v>
       </c>
       <c r="F37" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8.5999999999999993E-2</v>
       </c>
       <c r="G37" s="4">
@@ -4474,7 +3981,7 @@
         <v>4.7E-2</v>
       </c>
       <c r="F38" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.4E-2</v>
       </c>
       <c r="G38" s="4">
@@ -4567,7 +4074,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
       <c r="F39" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.9000000000000005E-2</v>
       </c>
       <c r="G39" s="4">
@@ -4660,7 +4167,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
       <c r="F40" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.9000000000000005E-2</v>
       </c>
       <c r="G40" s="4">
@@ -4753,7 +4260,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
       <c r="F41" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.9000000000000005E-2</v>
       </c>
       <c r="G41" s="4">
@@ -4846,7 +4353,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
       <c r="F42" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.9000000000000005E-2</v>
       </c>
       <c r="G42" s="4">
@@ -4939,7 +4446,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
       <c r="F43" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.9000000000000005E-2</v>
       </c>
       <c r="G43" s="4">
@@ -5032,7 +4539,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
       <c r="F44" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.9000000000000005E-2</v>
       </c>
       <c r="G44" s="4">
@@ -5125,7 +4632,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
       <c r="F45" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.9000000000000005E-2</v>
       </c>
       <c r="G45" s="4">
@@ -5218,7 +4725,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
       <c r="F46" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.9000000000000005E-2</v>
       </c>
       <c r="G46" s="4">
@@ -5311,7 +4818,7 @@
         <v>4.9500000000000002E-2</v>
       </c>
       <c r="F47" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>9.9000000000000005E-2</v>
       </c>
       <c r="G47" s="4">
@@ -5404,7 +4911,7 @@
         <v>5.0250000000000003E-2</v>
       </c>
       <c r="F48" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.10050000000000001</v>
       </c>
       <c r="G48" s="4">
@@ -5444,7 +4951,7 @@
         <v>453.49</v>
       </c>
       <c r="S48">
-        <v>2.7999999999999997E-2</v>
+        <v>2.8000000000000001E-2</v>
       </c>
       <c r="T48" s="2">
         <v>1</v>
@@ -5497,7 +5004,7 @@
         <v>5.0999999999999997E-2</v>
       </c>
       <c r="F49" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.10199999999999999</v>
       </c>
       <c r="G49" s="4">
@@ -5537,7 +5044,7 @@
         <v>457.57</v>
       </c>
       <c r="S49">
-        <v>1.8000000000000002E-2</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="T49" s="2">
         <v>1</v>
@@ -5590,7 +5097,7 @@
         <v>5.1749999999999997E-2</v>
       </c>
       <c r="F50" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.10349999999999999</v>
       </c>
       <c r="G50" s="4">
@@ -5683,7 +5190,7 @@
         <v>5.2499999999999998E-2</v>
       </c>
       <c r="F51" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.105</v>
       </c>
       <c r="G51" s="4">
@@ -5724,7 +5231,7 @@
         <v>471.4</v>
       </c>
       <c r="S51">
-        <v>1.8000000000000002E-2</v>
+        <v>1.7999999999999999E-2</v>
       </c>
       <c r="T51" s="2">
         <v>1</v>
@@ -5777,7 +5284,7 @@
         <v>5.3249999999999999E-2</v>
       </c>
       <c r="F52" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.1065</v>
       </c>
       <c r="G52" s="4">
@@ -5870,7 +5377,7 @@
         <v>5.3999999999999999E-2</v>
       </c>
       <c r="F53" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.108</v>
       </c>
       <c r="G53" s="4">
@@ -5910,7 +5417,7 @@
         <v>478</v>
       </c>
       <c r="S53">
-        <v>1.3999999999999999E-2</v>
+        <v>1.4E-2</v>
       </c>
       <c r="T53" s="2">
         <v>1</v>
@@ -5963,7 +5470,7 @@
         <v>5.3999999999999999E-2</v>
       </c>
       <c r="F54" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0.108</v>
       </c>
       <c r="G54" s="4">
@@ -6040,13 +5547,13 @@
       </c>
     </row>
     <row r="55" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A55" s="6">
+      <c r="A55" s="5">
         <v>2019</v>
       </c>
-      <c r="B55" s="9">
+      <c r="B55" s="6">
         <v>57400</v>
       </c>
-      <c r="C55" s="9">
+      <c r="C55" s="6">
         <v>3500</v>
       </c>
       <c r="D55" s="4">
@@ -6055,7 +5562,7 @@
       <c r="E55" s="4">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="F55" s="10">
+      <c r="F55" s="7">
         <v>0.108</v>
       </c>
       <c r="G55" s="4">
@@ -6064,46 +5571,46 @@
       <c r="H55" s="4">
         <v>0.06</v>
       </c>
-      <c r="I55" s="10">
+      <c r="I55" s="7">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="J55" s="9">
+      <c r="J55" s="6">
         <v>5</v>
       </c>
       <c r="K55" s="2">
         <v>0.25</v>
       </c>
-      <c r="L55" s="9">
+      <c r="L55" s="6">
         <v>0.15</v>
       </c>
-      <c r="M55" s="9">
+      <c r="M55" s="6">
         <v>60</v>
       </c>
-      <c r="N55" s="9">
-        <v>65</v>
-      </c>
-      <c r="O55" s="9">
+      <c r="N55" s="6">
+        <v>65</v>
+      </c>
+      <c r="O55" s="6">
         <v>70</v>
       </c>
       <c r="P55" s="3">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="Q55" s="9">
+      <c r="Q55" s="6">
         <v>0.75</v>
       </c>
-      <c r="R55" s="9">
+      <c r="R55" s="6">
         <v>496.33</v>
       </c>
-      <c r="S55" s="10">
+      <c r="S55" s="7">
         <v>2.3E-2</v>
       </c>
       <c r="T55" s="2">
         <v>1</v>
       </c>
-      <c r="U55" s="10">
+      <c r="U55" s="7">
         <v>1.5E-3</v>
       </c>
-      <c r="V55" s="10">
+      <c r="V55" s="7">
         <v>1.5E-3</v>
       </c>
       <c r="W55" s="2">
@@ -6112,16 +5619,16 @@
       <c r="X55" s="2">
         <v>0</v>
       </c>
-      <c r="Y55" s="10">
+      <c r="Y55" s="7">
         <v>3.0000000000000001E-3</v>
       </c>
       <c r="Z55" s="2">
         <v>0</v>
       </c>
-      <c r="AA55" s="11">
+      <c r="AA55" s="8">
         <v>8.3299999999999999E-2</v>
       </c>
-      <c r="AB55" s="11">
+      <c r="AB55" s="8">
         <v>0</v>
       </c>
       <c r="AC55" s="4">
@@ -6131,562 +5638,647 @@
         <v>6.6E-3</v>
       </c>
     </row>
-    <row r="56" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A56" s="6">
+    <row r="56" spans="1:30" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="10">
         <v>2020</v>
       </c>
-      <c r="B56" s="9">
+      <c r="B56" s="6">
         <v>58700</v>
       </c>
-      <c r="C56" s="9">
+      <c r="C56" s="6">
         <v>3500</v>
       </c>
-      <c r="D56" s="4">
+      <c r="D56" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="E56" s="4">
+      <c r="E56" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="F56" s="10">
+      <c r="F56" s="7">
         <v>0.108</v>
       </c>
-      <c r="G56" s="4">
+      <c r="G56" s="7">
         <v>1.2E-2</v>
       </c>
-      <c r="H56" s="4">
-        <v>0.06</v>
-      </c>
-      <c r="I56" s="10">
+      <c r="H56" s="7">
+        <v>0.06</v>
+      </c>
+      <c r="I56" s="7">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="J56" s="9">
+      <c r="J56" s="6">
         <v>5</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="6">
         <v>0.25</v>
       </c>
-      <c r="L56" s="9">
+      <c r="L56" s="6">
         <v>0.15</v>
       </c>
-      <c r="M56" s="9">
+      <c r="M56" s="6">
         <v>60</v>
       </c>
-      <c r="N56" s="9">
-        <v>65</v>
-      </c>
-      <c r="O56" s="9">
+      <c r="N56" s="6">
+        <v>65</v>
+      </c>
+      <c r="O56" s="6">
         <v>70</v>
       </c>
-      <c r="P56" s="3">
+      <c r="P56" s="8">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="Q56" s="9">
+      <c r="Q56" s="6">
         <v>0.75</v>
       </c>
-      <c r="R56" s="9">
+      <c r="R56" s="6">
         <v>505.76</v>
       </c>
-      <c r="S56" s="10">
+      <c r="S56" s="7">
         <v>1.9E-2</v>
       </c>
-      <c r="T56" s="2">
+      <c r="T56" s="6">
         <v>1</v>
       </c>
-      <c r="U56" s="10">
+      <c r="U56" s="7">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="V56" s="10">
+      <c r="V56" s="7">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="W56" s="2">
-        <v>0</v>
-      </c>
-      <c r="X56" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y56" s="10">
+      <c r="W56" s="6">
+        <v>0</v>
+      </c>
+      <c r="X56" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y56" s="7">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="Z56" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA56" s="11">
+      <c r="Z56" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA56" s="8">
         <v>8.3299999999999999E-2</v>
       </c>
-      <c r="AB56" s="11">
-        <v>0</v>
-      </c>
-      <c r="AC56" s="4">
+      <c r="AB56" s="8">
+        <v>0</v>
+      </c>
+      <c r="AC56" s="7">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="AD56" s="4">
+      <c r="AD56" s="7">
         <v>6.6E-3</v>
       </c>
     </row>
-    <row r="57" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A57" s="6">
+    <row r="57" spans="1:30" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="10">
         <v>2021</v>
       </c>
-      <c r="B57" s="9">
+      <c r="B57" s="6">
         <v>61600</v>
       </c>
-      <c r="C57" s="9">
+      <c r="C57" s="6">
         <v>3500</v>
       </c>
-      <c r="D57" s="4">
+      <c r="D57" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="E57" s="4">
+      <c r="E57" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="F57" s="4">
+      <c r="F57" s="7">
         <v>0.108</v>
       </c>
-      <c r="G57" s="4">
+      <c r="G57" s="7">
         <v>1.2E-2</v>
       </c>
-      <c r="H57" s="4">
-        <v>0.06</v>
-      </c>
-      <c r="I57" s="10">
+      <c r="H57" s="7">
+        <v>0.06</v>
+      </c>
+      <c r="I57" s="7">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="J57" s="9">
+      <c r="J57" s="6">
         <v>5</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="6">
         <v>0.25</v>
       </c>
-      <c r="L57" s="9">
+      <c r="L57" s="6">
         <v>0.15</v>
       </c>
-      <c r="M57" s="9">
+      <c r="M57" s="6">
         <v>60</v>
       </c>
-      <c r="N57" s="9">
-        <v>65</v>
-      </c>
-      <c r="O57" s="9">
+      <c r="N57" s="6">
+        <v>65</v>
+      </c>
+      <c r="O57" s="6">
         <v>70</v>
       </c>
-      <c r="P57" s="3">
+      <c r="P57" s="8">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="Q57" s="9">
+      <c r="Q57" s="6">
         <v>0.75</v>
       </c>
-      <c r="R57" s="9">
+      <c r="R57" s="6">
         <v>510.82</v>
       </c>
-      <c r="S57" s="10">
+      <c r="S57" s="7">
         <v>0.01</v>
       </c>
-      <c r="T57" s="2">
+      <c r="T57" s="6">
         <v>1</v>
       </c>
-      <c r="U57" s="10">
+      <c r="U57" s="7">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="V57" s="10">
+      <c r="V57" s="7">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="W57" s="2">
-        <v>0</v>
-      </c>
-      <c r="X57" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y57" s="10">
+      <c r="W57" s="6">
+        <v>0</v>
+      </c>
+      <c r="X57" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y57" s="7">
         <v>0.01</v>
       </c>
-      <c r="Z57" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA57" s="11">
+      <c r="Z57" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA57" s="8">
         <v>8.3299999999999999E-2</v>
       </c>
-      <c r="AB57" s="11">
-        <v>0</v>
-      </c>
-      <c r="AC57" s="4">
+      <c r="AB57" s="8">
+        <v>0</v>
+      </c>
+      <c r="AC57" s="7">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="AD57" s="4">
+      <c r="AD57" s="7">
         <v>6.6E-3</v>
       </c>
     </row>
-    <row r="58" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A58" s="6">
+    <row r="58" spans="1:30" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="10">
         <v>2022</v>
       </c>
-      <c r="B58" s="9">
+      <c r="B58" s="6">
         <v>64900</v>
       </c>
-      <c r="C58" s="9">
+      <c r="C58" s="6">
         <v>3500</v>
       </c>
-      <c r="D58" s="10">
+      <c r="D58" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="E58" s="10">
+      <c r="E58" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="F58" s="10">
+      <c r="F58" s="7">
         <v>0.108</v>
       </c>
-      <c r="G58" s="4">
+      <c r="G58" s="7">
         <v>1.2E-2</v>
       </c>
-      <c r="H58" s="4">
-        <v>0.06</v>
-      </c>
-      <c r="I58" s="8">
+      <c r="H58" s="7">
+        <v>0.06</v>
+      </c>
+      <c r="I58" s="7">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="J58" s="5">
+      <c r="J58" s="6">
         <v>5</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="6">
         <v>0.25</v>
       </c>
-      <c r="L58" s="9">
+      <c r="L58" s="6">
         <v>0.15</v>
       </c>
-      <c r="M58" s="5">
+      <c r="M58" s="6">
         <v>60</v>
       </c>
-      <c r="N58" s="5">
-        <v>65</v>
-      </c>
-      <c r="O58" s="5">
+      <c r="N58" s="6">
+        <v>65</v>
+      </c>
+      <c r="O58" s="6">
         <v>70</v>
       </c>
-      <c r="P58" s="3">
+      <c r="P58" s="8">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="Q58" s="5">
+      <c r="Q58" s="6">
         <v>0.75</v>
       </c>
-      <c r="R58" s="5">
-        <f t="shared" ref="R58:R61" si="1">R57*1.03</f>
-        <v>526.14459999999997</v>
-      </c>
-      <c r="S58" s="8">
-        <v>1.6750000000000001E-2</v>
-      </c>
-      <c r="T58" s="2">
+      <c r="R58" s="6">
+        <v>524.61</v>
+      </c>
+      <c r="S58" s="7">
+        <v>2.7E-2</v>
+      </c>
+      <c r="T58" s="6">
         <v>1</v>
       </c>
-      <c r="U58" s="10">
+      <c r="U58" s="7">
         <v>7.4999999999999997E-3</v>
       </c>
-      <c r="V58" s="10">
+      <c r="V58" s="7">
         <v>7.4999999999999997E-3</v>
       </c>
-      <c r="W58" s="2">
-        <v>0</v>
-      </c>
-      <c r="X58" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y58" s="11">
+      <c r="W58" s="6">
+        <v>0</v>
+      </c>
+      <c r="X58" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y58" s="8">
         <v>1.4999999999999999E-2</v>
       </c>
-      <c r="Z58" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA58" s="11">
+      <c r="Z58" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA58" s="8">
         <v>8.3299999999999999E-2</v>
       </c>
-      <c r="AB58" s="11">
-        <v>0</v>
-      </c>
-      <c r="AC58" s="4">
+      <c r="AB58" s="8">
+        <v>0</v>
+      </c>
+      <c r="AC58" s="7">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="AD58" s="4">
+      <c r="AD58" s="7">
         <v>6.6E-3</v>
       </c>
     </row>
-    <row r="59" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A59" s="6">
+    <row r="59" spans="1:30" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="10">
         <v>2023</v>
       </c>
-      <c r="B59" s="5">
-        <f t="shared" ref="B59:B61" si="2">B58*1.0159</f>
-        <v>65931.91</v>
-      </c>
-      <c r="C59" s="5">
+      <c r="B59" s="6">
+        <v>66600</v>
+      </c>
+      <c r="C59" s="6">
         <v>3500</v>
       </c>
-      <c r="D59" s="8">
+      <c r="D59" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="E59" s="8">
+      <c r="E59" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="F59" s="8">
+      <c r="F59" s="7">
         <v>0.108</v>
       </c>
-      <c r="G59" s="4">
+      <c r="G59" s="7">
         <v>1.2E-2</v>
       </c>
-      <c r="H59" s="4">
-        <v>0.06</v>
-      </c>
-      <c r="I59" s="8">
+      <c r="H59" s="7">
+        <v>0.06</v>
+      </c>
+      <c r="I59" s="7">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="J59" s="5">
+      <c r="J59" s="6">
         <v>5</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="6">
         <v>0.25</v>
       </c>
-      <c r="L59" s="5">
+      <c r="L59" s="6">
         <v>0.15</v>
       </c>
-      <c r="M59" s="5">
+      <c r="M59" s="6">
         <v>60</v>
       </c>
-      <c r="N59" s="5">
-        <v>65</v>
-      </c>
-      <c r="O59" s="5">
+      <c r="N59" s="6">
+        <v>65</v>
+      </c>
+      <c r="O59" s="6">
         <v>70</v>
       </c>
-      <c r="P59" s="3">
+      <c r="P59" s="8">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="Q59" s="5">
+      <c r="Q59" s="6">
         <v>0.75</v>
       </c>
-      <c r="R59" s="5">
-        <f t="shared" si="1"/>
-        <v>541.92893800000002</v>
-      </c>
-      <c r="S59" s="8">
-        <v>1.6750000000000001E-2</v>
-      </c>
-      <c r="T59" s="2">
+      <c r="R59" s="6">
+        <v>558.71</v>
+      </c>
+      <c r="S59" s="7">
+        <v>6.5000000000000002E-2</v>
+      </c>
+      <c r="T59" s="6">
         <v>1</v>
       </c>
-      <c r="U59" s="8">
+      <c r="U59" s="7">
         <v>0.01</v>
       </c>
-      <c r="V59" s="5">
+      <c r="V59" s="6">
         <v>0.01</v>
       </c>
-      <c r="W59" s="2">
-        <v>0</v>
-      </c>
-      <c r="X59" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y59" s="7">
+      <c r="W59" s="6">
+        <v>0</v>
+      </c>
+      <c r="X59" s="6">
+        <v>0</v>
+      </c>
+      <c r="Y59" s="8">
         <v>0.02</v>
       </c>
-      <c r="Z59" s="2">
-        <v>0</v>
-      </c>
-      <c r="AA59" s="11">
+      <c r="Z59" s="6">
+        <v>0</v>
+      </c>
+      <c r="AA59" s="8">
         <v>8.3299999999999999E-2</v>
       </c>
-      <c r="AB59" s="11">
-        <v>0</v>
-      </c>
-      <c r="AC59" s="4">
+      <c r="AB59" s="8">
+        <v>0</v>
+      </c>
+      <c r="AC59" s="7">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="AD59" s="4">
+      <c r="AD59" s="7">
         <v>6.6E-3</v>
       </c>
     </row>
-    <row r="60" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A60" s="6">
+    <row r="60" spans="1:30" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="10">
         <v>2024</v>
       </c>
-      <c r="B60" s="5">
-        <f t="shared" si="2"/>
-        <v>66980.227369</v>
-      </c>
-      <c r="C60" s="5">
+      <c r="B60" s="6">
+        <v>68500</v>
+      </c>
+      <c r="C60" s="6">
         <v>3500</v>
       </c>
-      <c r="D60" s="8">
+      <c r="D60" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="E60" s="8">
+      <c r="E60" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="F60" s="8">
+      <c r="F60" s="7">
         <v>0.108</v>
       </c>
-      <c r="G60" s="4">
+      <c r="G60" s="7">
         <v>1.2E-2</v>
       </c>
-      <c r="H60" s="4">
-        <v>0.06</v>
-      </c>
-      <c r="I60" s="8">
+      <c r="H60" s="7">
+        <v>0.06</v>
+      </c>
+      <c r="I60" s="7">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="J60" s="5">
+      <c r="J60" s="6">
         <v>5</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="6">
         <v>0.25</v>
       </c>
-      <c r="L60" s="5">
+      <c r="L60" s="6">
         <v>0.15</v>
       </c>
-      <c r="M60" s="5">
+      <c r="M60" s="6">
         <v>60</v>
       </c>
-      <c r="N60" s="5">
-        <v>65</v>
-      </c>
-      <c r="O60" s="5">
-        <v>70</v>
-      </c>
-      <c r="P60" s="3">
+      <c r="N60" s="6">
+        <v>65</v>
+      </c>
+      <c r="O60" s="6">
+        <v>72</v>
+      </c>
+      <c r="P60" s="8">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="Q60" s="5">
+      <c r="Q60" s="6">
         <v>0.75</v>
       </c>
-      <c r="R60" s="5">
-        <f t="shared" si="1"/>
-        <v>558.18680614000004</v>
-      </c>
-      <c r="S60" s="8">
-        <v>1.6750000000000001E-2</v>
-      </c>
-      <c r="T60" s="5">
-        <v>1.07</v>
-      </c>
-      <c r="U60" s="8">
+      <c r="R60" s="6">
+        <v>583.29</v>
+      </c>
+      <c r="S60" s="7">
+        <v>4.3999999999999997E-2</v>
+      </c>
+      <c r="T60" s="6">
+        <v>1.06861313869</v>
+      </c>
+      <c r="U60" s="7">
         <v>0.01</v>
       </c>
-      <c r="V60" s="5">
+      <c r="V60" s="6">
         <v>0.01</v>
       </c>
-      <c r="W60" s="5">
+      <c r="W60" s="6">
         <v>0.04</v>
       </c>
-      <c r="X60" s="5">
+      <c r="X60" s="6">
         <v>0.04</v>
       </c>
-      <c r="Y60" s="7">
+      <c r="Y60" s="8">
         <v>0.02</v>
       </c>
-      <c r="Z60" s="5">
+      <c r="Z60" s="6">
         <v>0.08</v>
       </c>
-      <c r="AA60" s="11">
+      <c r="AA60" s="8">
         <v>8.3299999999999999E-2</v>
       </c>
-      <c r="AB60" s="11">
+      <c r="AB60" s="8">
         <v>0.33329999999999999</v>
       </c>
-      <c r="AC60" s="4">
+      <c r="AC60" s="7">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="AD60" s="4">
+      <c r="AD60" s="7">
         <v>6.6E-3</v>
       </c>
     </row>
-    <row r="61" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="A61" s="6">
+    <row r="61" spans="1:30" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="10">
         <v>2025</v>
       </c>
-      <c r="B61" s="5">
-        <f t="shared" si="2"/>
-        <v>68045.212984167098</v>
-      </c>
-      <c r="C61" s="5">
+      <c r="B61" s="6">
+        <v>71300</v>
+      </c>
+      <c r="C61" s="6">
         <v>3500</v>
       </c>
-      <c r="D61" s="8">
+      <c r="D61" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="E61" s="8">
+      <c r="E61" s="7">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="F61" s="8">
+      <c r="F61" s="7">
         <v>0.108</v>
       </c>
-      <c r="G61" s="4">
+      <c r="G61" s="7">
         <v>1.2E-2</v>
       </c>
-      <c r="H61" s="4">
-        <v>0.06</v>
-      </c>
-      <c r="I61" s="8">
+      <c r="H61" s="7">
+        <v>0.06</v>
+      </c>
+      <c r="I61" s="7">
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="J61" s="5">
+      <c r="J61" s="6">
         <v>5</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="6">
         <v>0.25</v>
       </c>
-      <c r="L61" s="5">
+      <c r="L61" s="6">
         <v>0.15</v>
       </c>
-      <c r="M61" s="5">
+      <c r="M61" s="6">
         <v>60</v>
       </c>
-      <c r="N61" s="5">
-        <v>65</v>
-      </c>
-      <c r="O61" s="5">
-        <v>70</v>
-      </c>
-      <c r="P61" s="3">
+      <c r="N61" s="6">
+        <v>65</v>
+      </c>
+      <c r="O61" s="6">
+        <v>72</v>
+      </c>
+      <c r="P61" s="8">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="Q61" s="5">
+      <c r="Q61" s="6">
         <v>0.75</v>
       </c>
-      <c r="R61" s="5">
-        <f t="shared" si="1"/>
-        <v>574.93241032420008</v>
-      </c>
-      <c r="S61" s="8">
-        <v>1.6750000000000001E-2</v>
-      </c>
-      <c r="T61" s="5">
-        <v>1.1399999999999999</v>
-      </c>
-      <c r="U61" s="8">
+      <c r="R61" s="6">
+        <v>598.46</v>
+      </c>
+      <c r="S61" s="7">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="T61" s="6">
+        <v>1.1388499298700001</v>
+      </c>
+      <c r="U61" s="7">
         <v>0.01</v>
       </c>
-      <c r="V61" s="5">
+      <c r="V61" s="6">
         <v>0.01</v>
       </c>
-      <c r="W61" s="5">
+      <c r="W61" s="6">
         <v>0.04</v>
       </c>
-      <c r="X61" s="5">
+      <c r="X61" s="6">
         <v>0.04</v>
       </c>
-      <c r="Y61" s="7">
+      <c r="Y61" s="8">
         <v>0.02</v>
       </c>
-      <c r="Z61" s="5">
+      <c r="Z61" s="6">
         <v>0.08</v>
       </c>
-      <c r="AA61" s="11">
+      <c r="AA61" s="8">
         <v>8.3299999999999999E-2</v>
       </c>
-      <c r="AB61" s="11">
+      <c r="AB61" s="8">
         <v>0.33329999999999999</v>
       </c>
-      <c r="AC61" s="4">
+      <c r="AC61" s="7">
         <v>1.6000000000000001E-3</v>
       </c>
-      <c r="AD61" s="4">
+      <c r="AD61" s="7">
+        <v>6.6E-3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:30" x14ac:dyDescent="0.25">
+      <c r="A62" s="10">
+        <v>2026</v>
+      </c>
+      <c r="B62" s="6">
+        <v>74600</v>
+      </c>
+      <c r="C62" s="6">
+        <v>3500</v>
+      </c>
+      <c r="D62" s="7">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="E62" s="7">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="F62" s="7">
+        <v>0.106</v>
+      </c>
+      <c r="G62" s="7">
+        <v>1.2E-2</v>
+      </c>
+      <c r="H62" s="7">
+        <v>0.06</v>
+      </c>
+      <c r="I62" s="7">
+        <v>8.4000000000000005E-2</v>
+      </c>
+      <c r="J62" s="6">
+        <v>5</v>
+      </c>
+      <c r="K62" s="6">
+        <v>0.25</v>
+      </c>
+      <c r="L62" s="6">
+        <v>0.15</v>
+      </c>
+      <c r="M62" s="6">
+        <v>60</v>
+      </c>
+      <c r="N62" s="6">
+        <v>65</v>
+      </c>
+      <c r="O62" s="6">
+        <v>72</v>
+      </c>
+      <c r="P62" s="8">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="Q62" s="6">
+        <v>0.75</v>
+      </c>
+      <c r="R62" s="6">
+        <v>610.42999999999995</v>
+      </c>
+      <c r="S62" s="7">
+        <v>0.02</v>
+      </c>
+      <c r="T62" s="6">
+        <v>1.13941018766756</v>
+      </c>
+      <c r="U62" s="7">
+        <v>0.01</v>
+      </c>
+      <c r="V62" s="6">
+        <v>0.01</v>
+      </c>
+      <c r="W62" s="6">
+        <v>0.04</v>
+      </c>
+      <c r="X62" s="6">
+        <v>0.04</v>
+      </c>
+      <c r="Y62" s="8">
+        <v>0.02</v>
+      </c>
+      <c r="Z62" s="6">
+        <v>0.08</v>
+      </c>
+      <c r="AA62" s="8">
+        <v>8.3299999999999999E-2</v>
+      </c>
+      <c r="AB62" s="8">
+        <v>0.33329999999999999</v>
+      </c>
+      <c r="AC62" s="7">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="AD62" s="7">
         <v>6.6E-3</v>
       </c>
     </row>

</xml_diff>